<commit_message>
KLEE test suite: reworked open test suite + excel changes
</commit_message>
<xml_diff>
--- a/individual_Tests/dup/dup_test_results.xlsx
+++ b/individual_Tests/dup/dup_test_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Masters\Tests\initial_tests\individual_Tests\dup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF493D7-7FEA-43C8-B08F-DE6A7D7F7565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05244726-1454-449F-B71E-90ED3845C85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11340" yWindow="6300" windowWidth="18345" windowHeight="8760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dup dup2 Test Results" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="76">
   <si>
     <t>Test ID</t>
   </si>

</xml_diff>